<commit_message>
Completado el approach de los q-gramas y distancias de leversney
</commit_message>
<xml_diff>
--- a/sandbox/tablas_locales_CC/direccion_centros_comerciales.xlsx
+++ b/sandbox/tablas_locales_CC/direccion_centros_comerciales.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atiscodesa-my.sharepoint.com/personal/ruben_freire_centrohub_co/Documents/Escritorio/Proyectos/CENTROS COMERCIALES/sandbox/tablas_locales_CC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_B8923127FC392AD0CAA53CFA5F3D01394A199D78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D1A670E-32DF-4845-A62F-9CD78E41C04E}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_B8923127FC392AD0CAA53CFA5F3D01394A199D78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05FC5FFB-75AD-492A-9821-03D240B3D7B0}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="20" windowWidth="19180" windowHeight="11260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$G$72</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -680,13 +683,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G72"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="36.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.88671875" customWidth="1"/>
+    <col min="3" max="3" width="25.5546875" customWidth="1"/>
+    <col min="6" max="6" width="30.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -709,7 +716,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -732,7 +739,7 @@
         <v>138.40823392473499</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -755,7 +762,7 @@
         <v>540.67023089133102</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -778,7 +785,7 @@
         <v>325.791437829492</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -801,7 +808,7 @@
         <v>142.68839364873099</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -824,7 +831,7 @@
         <v>290.66136985165502</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -847,7 +854,7 @@
         <v>602.11897703683599</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -870,7 +877,7 @@
         <v>111.680588462207</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -893,7 +900,7 @@
         <v>311.07325456247099</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -916,7 +923,7 @@
         <v>1158.70064695883</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -939,7 +946,7 @@
         <v>196.714745745594</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -962,7 +969,7 @@
         <v>199.285464767473</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -985,7 +992,7 @@
         <v>330.375503224672</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1008,7 +1015,7 @@
         <v>580.28175310349104</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1031,7 +1038,7 @@
         <v>285.771853392683</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1054,7 +1061,7 @@
         <v>45.977889404214103</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1077,7 +1084,7 @@
         <v>234.60037123497099</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -1100,7 +1107,7 @@
         <v>159.94738968603701</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1123,7 +1130,7 @@
         <v>96.962074256819307</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -1146,7 +1153,7 @@
         <v>384.413312659366</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1169,7 +1176,7 @@
         <v>31.049061264116901</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -1192,7 +1199,7 @@
         <v>117.286311903759</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -1215,7 +1222,7 @@
         <v>136.030620273735</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1238,7 +1245,7 @@
         <v>148.563737943283</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -1261,7 +1268,7 @@
         <v>168.57044375472401</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -1284,7 +1291,7 @@
         <v>178.992709472359</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1307,7 +1314,7 @@
         <v>102.98955628349501</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1330,7 +1337,7 @@
         <v>141.263068625416</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>51</v>
       </c>
@@ -1353,7 +1360,7 @@
         <v>391.54785761813997</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>51</v>
       </c>
@@ -1376,7 +1383,7 @@
         <v>381.05599828641698</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>51</v>
       </c>
@@ -1399,7 +1406,7 @@
         <v>162.973507280918</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -1422,7 +1429,7 @@
         <v>351.97873005499702</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>51</v>
       </c>
@@ -1445,7 +1452,7 @@
         <v>394.04605779158499</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -1468,7 +1475,7 @@
         <v>699.22581497090698</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>55</v>
       </c>
@@ -1491,7 +1498,7 @@
         <v>32.224679898874598</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>55</v>
       </c>
@@ -1514,7 +1521,7 @@
         <v>62.811542017962303</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>55</v>
       </c>
@@ -1537,7 +1544,7 @@
         <v>340.38020009252</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>55</v>
       </c>
@@ -1560,7 +1567,7 @@
         <v>624.07879155470903</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>62</v>
       </c>
@@ -1583,7 +1590,7 @@
         <v>73.757182716534899</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>62</v>
       </c>
@@ -1606,7 +1613,7 @@
         <v>808.52064006190199</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -1629,7 +1636,7 @@
         <v>357.79974948821598</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>62</v>
       </c>
@@ -1652,7 +1659,7 @@
         <v>207.66727657583101</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>68</v>
       </c>
@@ -1675,7 +1682,7 @@
         <v>262.97786250478498</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>68</v>
       </c>
@@ -1698,7 +1705,7 @@
         <v>169.28446927254799</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>68</v>
       </c>
@@ -1721,7 +1728,7 @@
         <v>240.32080747259599</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>68</v>
       </c>
@@ -1744,7 +1751,7 @@
         <v>282.00151498121301</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>75</v>
       </c>
@@ -1767,7 +1774,7 @@
         <v>614.78921064085898</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>75</v>
       </c>
@@ -1790,7 +1797,7 @@
         <v>373.59095652266097</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>75</v>
       </c>
@@ -1813,7 +1820,7 @@
         <v>65.302105335114206</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>75</v>
       </c>
@@ -1836,7 +1843,7 @@
         <v>281.38181072059302</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>79</v>
       </c>
@@ -1859,7 +1866,7 @@
         <v>231.242741333071</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>79</v>
       </c>
@@ -1882,7 +1889,7 @@
         <v>457.93714437890799</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>79</v>
       </c>
@@ -1905,7 +1912,7 @@
         <v>38.858925300894903</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>79</v>
       </c>
@@ -1928,7 +1935,7 @@
         <v>80.351302825920499</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>79</v>
       </c>
@@ -1951,7 +1958,7 @@
         <v>225.44532421382399</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>86</v>
       </c>
@@ -1974,7 +1981,7 @@
         <v>90.931574337918605</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>86</v>
       </c>
@@ -1997,7 +2004,7 @@
         <v>184.71347926132799</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>86</v>
       </c>
@@ -2020,7 +2027,7 @@
         <v>171.80313394621299</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>86</v>
       </c>
@@ -2043,7 +2050,7 @@
         <v>197.29867817240401</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>86</v>
       </c>
@@ -2066,7 +2073,7 @@
         <v>51.909959632089297</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>94</v>
       </c>
@@ -2089,7 +2096,7 @@
         <v>261.92013720277401</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>94</v>
       </c>
@@ -2112,7 +2119,7 @@
         <v>217.338125422226</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>94</v>
       </c>
@@ -2135,7 +2142,7 @@
         <v>449.70613862033599</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>100</v>
       </c>
@@ -2158,7 +2165,7 @@
         <v>162.234575689975</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>100</v>
       </c>
@@ -2181,7 +2188,7 @@
         <v>261.07131247795598</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>100</v>
       </c>
@@ -2204,7 +2211,7 @@
         <v>354.83623993461498</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>100</v>
       </c>
@@ -2227,7 +2234,7 @@
         <v>386.88334970749003</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>104</v>
       </c>
@@ -2250,7 +2257,7 @@
         <v>226.92603327882199</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>104</v>
       </c>
@@ -2273,7 +2280,7 @@
         <v>169.494198074531</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>106</v>
       </c>
@@ -2296,7 +2303,7 @@
         <v>619.24788519907895</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>106</v>
       </c>
@@ -2319,7 +2326,7 @@
         <v>34.651812886220199</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>106</v>
       </c>
@@ -2343,6 +2350,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G72" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="CENTRO COMERCIAL CONDADO SHOPPING"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
añadir columna a la tabla consolidacion master
</commit_message>
<xml_diff>
--- a/sandbox/tablas_locales_CC/direccion_centros_comerciales.xlsx
+++ b/sandbox/tablas_locales_CC/direccion_centros_comerciales.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atiscodesa-my.sharepoint.com/personal/ruben_freire_centrohub_co/Documents/Escritorio/Proyectos/CENTROS COMERCIALES/sandbox/tablas_locales_CC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_B8923127FC392AD0CAA53CFA5F3D01394A199D78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{05FC5FFB-75AD-492A-9821-03D240B3D7B0}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="11_B8923127FC392AD0CAA53CFA5F3D01394A199D78" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9FD9E0B-673E-4207-9ECB-356022DAD10F}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="24" windowWidth="23016" windowHeight="12216" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
@@ -683,13 +683,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.88671875" customWidth="1"/>
-    <col min="3" max="3" width="25.5546875" customWidth="1"/>
+    <col min="3" max="3" width="44.6640625" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
     <col min="6" max="6" width="30.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -831,7 +831,7 @@
         <v>290.66136985165502</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -854,7 +854,7 @@
         <v>602.11897703683599</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -877,7 +877,7 @@
         <v>111.680588462207</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -900,7 +900,7 @@
         <v>311.07325456247099</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -923,7 +923,7 @@
         <v>1158.70064695883</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -946,7 +946,7 @@
         <v>196.714745745594</v>
       </c>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -969,7 +969,7 @@
         <v>199.285464767473</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -992,7 +992,7 @@
         <v>330.375503224672</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1015,7 +1015,7 @@
         <v>580.28175310349104</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>29</v>
       </c>
@@ -1038,7 +1038,7 @@
         <v>285.771853392683</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>45.977889404214103</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>29</v>
       </c>
@@ -1084,7 +1084,7 @@
         <v>234.60037123497099</v>
       </c>
     </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>29</v>
       </c>
@@ -1107,7 +1107,7 @@
         <v>159.94738968603701</v>
       </c>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>37</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>96.962074256819307</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>37</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>384.413312659366</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>37</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>31.049061264116901</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>37</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>117.286311903759</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>136.030620273735</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1245,7 +1245,7 @@
         <v>148.563737943283</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -1268,7 +1268,7 @@
         <v>168.57044375472401</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -1291,7 +1291,7 @@
         <v>178.992709472359</v>
       </c>
     </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>102.98955628349501</v>
       </c>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1337,7 +1337,7 @@
         <v>141.263068625416</v>
       </c>
     </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>51</v>
       </c>
@@ -1360,7 +1360,7 @@
         <v>391.54785761813997</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>51</v>
       </c>
@@ -1383,7 +1383,7 @@
         <v>381.05599828641698</v>
       </c>
     </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>51</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>162.973507280918</v>
       </c>
     </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>51</v>
       </c>
@@ -1429,7 +1429,7 @@
         <v>351.97873005499702</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>51</v>
       </c>
@@ -1452,7 +1452,7 @@
         <v>394.04605779158499</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -1475,7 +1475,7 @@
         <v>699.22581497090698</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>55</v>
       </c>
@@ -1498,7 +1498,7 @@
         <v>32.224679898874598</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>55</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>62.811542017962303</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>55</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>340.38020009252</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>55</v>
       </c>
@@ -1567,7 +1567,7 @@
         <v>624.07879155470903</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>62</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>73.757182716534899</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>62</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>808.52064006190199</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>62</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>357.79974948821598</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>62</v>
       </c>
@@ -1659,7 +1659,7 @@
         <v>207.66727657583101</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>68</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>262.97786250478498</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>68</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>169.28446927254799</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>68</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>240.32080747259599</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>68</v>
       </c>
@@ -1751,7 +1751,7 @@
         <v>282.00151498121301</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>75</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>614.78921064085898</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>75</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>373.59095652266097</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>75</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>65.302105335114206</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>75</v>
       </c>
@@ -1843,7 +1843,7 @@
         <v>281.38181072059302</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>79</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>231.242741333071</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>79</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>457.93714437890799</v>
       </c>
     </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>79</v>
       </c>
@@ -1912,7 +1912,7 @@
         <v>38.858925300894903</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>79</v>
       </c>
@@ -1935,7 +1935,7 @@
         <v>80.351302825920499</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>79</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>225.44532421382399</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>86</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>90.931574337918605</v>
       </c>
     </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>86</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>184.71347926132799</v>
       </c>
     </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>86</v>
       </c>
@@ -2027,7 +2027,7 @@
         <v>171.80313394621299</v>
       </c>
     </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>86</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>197.29867817240401</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>86</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>51.909959632089297</v>
       </c>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>94</v>
       </c>
@@ -2096,7 +2096,7 @@
         <v>261.92013720277401</v>
       </c>
     </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>94</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>217.338125422226</v>
       </c>
     </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>94</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>449.70613862033599</v>
       </c>
     </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>100</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>162.234575689975</v>
       </c>
     </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>100</v>
       </c>
@@ -2188,7 +2188,7 @@
         <v>261.07131247795598</v>
       </c>
     </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>100</v>
       </c>
@@ -2211,7 +2211,7 @@
         <v>354.83623993461498</v>
       </c>
     </row>
-    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>100</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>386.88334970749003</v>
       </c>
     </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>104</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>226.92603327882199</v>
       </c>
     </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>104</v>
       </c>
@@ -2280,7 +2280,7 @@
         <v>169.494198074531</v>
       </c>
     </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>106</v>
       </c>
@@ -2303,7 +2303,7 @@
         <v>619.24788519907895</v>
       </c>
     </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>106</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>34.651812886220199</v>
       </c>
     </row>
-    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>106</v>
       </c>
@@ -2350,13 +2350,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G72" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="CENTRO COMERCIAL CONDADO SHOPPING"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G72" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>